<commit_message>
Added birds of Americas.
</commit_message>
<xml_diff>
--- a/i18n/template.xlsx
+++ b/i18n/template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Birds" sheetId="1" state="visible" r:id="rId3"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1574" uniqueCount="1021">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1907" uniqueCount="1244">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -2753,6 +2753,675 @@
   </si>
   <si>
     <t xml:space="preserve">Geopelia striata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barred Antshrike</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thamophilus doliatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">americas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bananaquit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coereba flaveola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antioquia Brushfinch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atlapetes blancae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altamira Oriole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Icterus gularis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazon Kingfisher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chloroceryle amazona</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazonian Parrotlet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nannopsittaca dachilleae</t>
+  </si>
+  <si>
+    <t xml:space="preserve">American Flamingo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phoenicopterus ruber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">American Golden-Plover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pluvialis dominica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andean Cock-of-the-Rock</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rupicola peruvianus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andean Condor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vultur gryphus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bat Falcon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falco rufigularis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black Rail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laterallus jamaicensis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue-Black Grassquit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volatinia jacarina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue-Footed Booby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sula nebouxii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue-Grey Tanager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thraupis episcopus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue-Headed Parrot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pionus menstruus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue-and-Yellow Macaw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ara ararauna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boat-Billed Heron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cochlearius cochlearius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brazilian Merganser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mergus octosetaceus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brazilian Teal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amazonetta brasiliensis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chiloé Wigeon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mareca sibilatrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clay-Colored Thrush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turdus grayi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cocoi Heron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ardea cocoi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Common Pauraque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nyctidromus albicollis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correndera Pipit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anthus correndera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crested Oropendola</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Psarocolius decumanus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elegant Trogon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trogon elegans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ferruginous Pygmy-Owl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glaucidium brasilianum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firewood-Gatherer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Anumbius annumbi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Golden-Headed Manakin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ceratopipra erythrocephala</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grassland Sparrow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ammodramus humeralis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Great Curassow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crax rubra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Great Kiskadee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pitangus sulphuratus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Great Potoo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nyctibius grandis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Great-Tailed Grackle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quiscalus mexicanus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greater Rhea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rhea americana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harpy Eagle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harpia harpyja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoatzin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opisthocomus hoazin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hooded Siskin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spinus magellanicus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Horned Guan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oreophasis derbianus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inca Tern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Larosterna inca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jabiru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jabiru mycteria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keel-Billed Toucan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ramphastos sulfuratus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">King Vulture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sarcoramphus papa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Least Seedsnipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thinocorus rumicivorus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limpkin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aramus guarauna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lineated Woodpecker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dryocopus lineatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Little Blue Heron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Egretta caerulea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Little Tinamou</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crypturellus soui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long-Wattled Umbrellabird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cephalopterus penduliger</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Magnificent Frigatebird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fregata magnificens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marsh Seedeater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sporophila palustris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monk Parakett</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Myiopsitta monachus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muscovy Duck</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cairina moschata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nanday Parakett</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aratinga nenday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neotropic Cormorant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nannopterum brasilianum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ocellated Turkey</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meleagris ocellata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oilbird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steastornis caripensis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orange-Breated Bunting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passerina leclancherii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orinoco Goose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neochen jubata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paradise Tanager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tangara chilensis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peruvian Sierra-Finch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phrygilus punensis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plain Chachalaca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ortalis vetula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red-Billed Scythebill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campylorhampus trochilirostris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red-Breated Meadowlark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leistes militaris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red-Crested Cardinal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paraoaria coronata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red-Headed Barbet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eubucco bourcierii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Red-Legged Seriema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cariama cristata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resplendent Quetzal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pharomachrus mocinno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roadside Hawk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rupornis magnirostris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ruddy Ground Dove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columbina talpacoti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rufescent Tiger-Heron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tigrisoma lineatum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rufous Hornero</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Furnarius rufus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rufous-Collared Sparrow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zonotrichia capensis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rufous-Naped Wren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campylorhampus rufinucha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Savanna Hawk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Butogallus meridionalis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scarlet Ibis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eudocimus ruber</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scarlet Macaw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ara macao</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Screaming Piha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lipaugus vociferans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shiny Cowbird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Molothrus bonariensis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smooth-Billed Ani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crotophaga ani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snowy Albatross</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diomedea exulans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southern Lapwing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vanellus chilensis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southern Rough-Winged Swallow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stelgidopteryx ruficollis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southern Screamer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chauna Torquata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spectacled Owl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pulsatrix perspicillata</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotted Nothura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nothura maulosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spotted Puffbird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bucco tamatia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Squirrel Cuckoo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piaya cayana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strange-Tailed Tyrant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alectrurus risora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun Parakett</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aratinga solstitialis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunbittern</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eurypyga helias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sungrebe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heliornis fulica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titicaca Grebe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rollandia microptera</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toco Toucan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ramphastos toco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tropical Kingbird</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tyrannyus melancholicus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tropical Parula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setophaga pitiayumi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tropical Royal Flycatcher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Onychorhynchus coronatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Turquisoe-Browed Motmot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eumomota superciliosa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ultramarine Grosbreak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyanoloxia brissonii</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vampire Ground-Finch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Geopspiza septentrionalis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable Seedeater</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sporophila corvina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verdin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auriparus flaviceps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vermillion Flycatcher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puyrocephalus rubinus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wattled Jacana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jacana jacana</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Western Rockhopper Penguin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eudyotes chrysocome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White-Browed Tit-Spinetail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leptasthenura xenothorax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White-Throated Magpie-Jay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyanocorax formosus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">White-Tipped Dove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leptotila verreauxi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow Warbler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Setophaga petechia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yellow-Headed Caracara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daptrius chimachima</t>
   </si>
   <si>
     <t xml:space="preserve">Name</t>
@@ -3325,37 +3994,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546a"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e7e6e6"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5b9bd5"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ed7d31"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a5a5a5"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="ffc000"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472c4"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70ad47"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563c1"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954f72"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -3494,7 +4163,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K447"/>
+  <dimension ref="A1:K1048576"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4.44"/>
@@ -10176,6 +10845,1563 @@
         <v>729</v>
       </c>
     </row>
+    <row r="448" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A448" s="1" t="n">
+        <v>607</v>
+      </c>
+      <c r="B448" s="1" t="s">
+        <v>908</v>
+      </c>
+      <c r="C448" s="1" t="s">
+        <v>909</v>
+      </c>
+      <c r="D448" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="449" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A449" s="1" t="n">
+        <v>606</v>
+      </c>
+      <c r="B449" s="1" t="s">
+        <v>911</v>
+      </c>
+      <c r="C449" s="1" t="s">
+        <v>912</v>
+      </c>
+      <c r="D449" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="450" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A450" s="1" t="n">
+        <v>605</v>
+      </c>
+      <c r="B450" s="1" t="s">
+        <v>913</v>
+      </c>
+      <c r="C450" s="1" t="s">
+        <v>914</v>
+      </c>
+      <c r="D450" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="451" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A451" s="1" t="n">
+        <v>598</v>
+      </c>
+      <c r="B451" s="1" t="s">
+        <v>915</v>
+      </c>
+      <c r="C451" s="1" t="s">
+        <v>916</v>
+      </c>
+      <c r="D451" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="452" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A452" s="1" t="n">
+        <v>599</v>
+      </c>
+      <c r="B452" s="1" t="s">
+        <v>917</v>
+      </c>
+      <c r="C452" s="1" t="s">
+        <v>918</v>
+      </c>
+      <c r="D452" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="453" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A453" s="1" t="n">
+        <v>600</v>
+      </c>
+      <c r="B453" s="1" t="s">
+        <v>919</v>
+      </c>
+      <c r="C453" s="1" t="s">
+        <v>920</v>
+      </c>
+      <c r="D453" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="454" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A454" s="1" t="n">
+        <v>601</v>
+      </c>
+      <c r="B454" s="1" t="s">
+        <v>921</v>
+      </c>
+      <c r="C454" s="1" t="s">
+        <v>922</v>
+      </c>
+      <c r="D454" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="455" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A455" s="1" t="n">
+        <v>602</v>
+      </c>
+      <c r="B455" s="1" t="s">
+        <v>923</v>
+      </c>
+      <c r="C455" s="1" t="s">
+        <v>924</v>
+      </c>
+      <c r="D455" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="456" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A456" s="1" t="n">
+        <v>603</v>
+      </c>
+      <c r="B456" s="1" t="s">
+        <v>925</v>
+      </c>
+      <c r="C456" s="1" t="s">
+        <v>926</v>
+      </c>
+      <c r="D456" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="457" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A457" s="1" t="n">
+        <v>604</v>
+      </c>
+      <c r="B457" s="1" t="s">
+        <v>927</v>
+      </c>
+      <c r="C457" s="1" t="s">
+        <v>928</v>
+      </c>
+      <c r="D457" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="458" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A458" s="1" t="n">
+        <v>608</v>
+      </c>
+      <c r="B458" s="1" t="s">
+        <v>929</v>
+      </c>
+      <c r="C458" s="1" t="s">
+        <v>930</v>
+      </c>
+      <c r="D458" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="459" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A459" s="1" t="n">
+        <v>609</v>
+      </c>
+      <c r="B459" s="1" t="s">
+        <v>931</v>
+      </c>
+      <c r="C459" s="1" t="s">
+        <v>932</v>
+      </c>
+      <c r="D459" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="460" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A460" s="1" t="n">
+        <v>610</v>
+      </c>
+      <c r="B460" s="1" t="s">
+        <v>933</v>
+      </c>
+      <c r="C460" s="1" t="s">
+        <v>934</v>
+      </c>
+      <c r="D460" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="461" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A461" s="1" t="n">
+        <v>611</v>
+      </c>
+      <c r="B461" s="1" t="s">
+        <v>935</v>
+      </c>
+      <c r="C461" s="1" t="s">
+        <v>936</v>
+      </c>
+      <c r="D461" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="462" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A462" s="1" t="n">
+        <v>612</v>
+      </c>
+      <c r="B462" s="1" t="s">
+        <v>937</v>
+      </c>
+      <c r="C462" s="1" t="s">
+        <v>938</v>
+      </c>
+      <c r="D462" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="463" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A463" s="1" t="n">
+        <v>613</v>
+      </c>
+      <c r="B463" s="1" t="s">
+        <v>939</v>
+      </c>
+      <c r="C463" s="1" t="s">
+        <v>940</v>
+      </c>
+      <c r="D463" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="464" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A464" s="1" t="n">
+        <v>614</v>
+      </c>
+      <c r="B464" s="1" t="s">
+        <v>941</v>
+      </c>
+      <c r="C464" s="1" t="s">
+        <v>942</v>
+      </c>
+      <c r="D464" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="465" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A465" s="1" t="n">
+        <v>615</v>
+      </c>
+      <c r="B465" s="1" t="s">
+        <v>943</v>
+      </c>
+      <c r="C465" s="1" t="s">
+        <v>944</v>
+      </c>
+      <c r="D465" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="466" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A466" s="1" t="n">
+        <v>616</v>
+      </c>
+      <c r="B466" s="1" t="s">
+        <v>945</v>
+      </c>
+      <c r="C466" s="1" t="s">
+        <v>946</v>
+      </c>
+      <c r="D466" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="467" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A467" s="1" t="n">
+        <v>617</v>
+      </c>
+      <c r="B467" s="1" t="s">
+        <v>947</v>
+      </c>
+      <c r="C467" s="1" t="s">
+        <v>948</v>
+      </c>
+      <c r="D467" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="468" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A468" s="1" t="n">
+        <v>618</v>
+      </c>
+      <c r="B468" s="1" t="s">
+        <v>949</v>
+      </c>
+      <c r="C468" s="1" t="s">
+        <v>950</v>
+      </c>
+      <c r="D468" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="469" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A469" s="1" t="n">
+        <v>619</v>
+      </c>
+      <c r="B469" s="1" t="s">
+        <v>951</v>
+      </c>
+      <c r="C469" s="1" t="s">
+        <v>952</v>
+      </c>
+      <c r="D469" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="470" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A470" s="1" t="n">
+        <v>620</v>
+      </c>
+      <c r="B470" s="1" t="s">
+        <v>953</v>
+      </c>
+      <c r="C470" s="1" t="s">
+        <v>954</v>
+      </c>
+      <c r="D470" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="471" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A471" s="1" t="n">
+        <v>621</v>
+      </c>
+      <c r="B471" s="1" t="s">
+        <v>955</v>
+      </c>
+      <c r="C471" s="1" t="s">
+        <v>956</v>
+      </c>
+      <c r="D471" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="472" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A472" s="1" t="n">
+        <v>622</v>
+      </c>
+      <c r="B472" s="1" t="s">
+        <v>957</v>
+      </c>
+      <c r="C472" s="1" t="s">
+        <v>958</v>
+      </c>
+      <c r="D472" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="473" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A473" s="1" t="n">
+        <v>623</v>
+      </c>
+      <c r="B473" s="1" t="s">
+        <v>959</v>
+      </c>
+      <c r="C473" s="1" t="s">
+        <v>960</v>
+      </c>
+      <c r="D473" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="474" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A474" s="1" t="n">
+        <v>624</v>
+      </c>
+      <c r="B474" s="1" t="s">
+        <v>961</v>
+      </c>
+      <c r="C474" s="1" t="s">
+        <v>962</v>
+      </c>
+      <c r="D474" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="475" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A475" s="1" t="n">
+        <v>625</v>
+      </c>
+      <c r="B475" s="1" t="s">
+        <v>963</v>
+      </c>
+      <c r="C475" s="1" t="s">
+        <v>964</v>
+      </c>
+      <c r="D475" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="476" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A476" s="1" t="n">
+        <v>626</v>
+      </c>
+      <c r="B476" s="1" t="s">
+        <v>965</v>
+      </c>
+      <c r="C476" s="1" t="s">
+        <v>966</v>
+      </c>
+      <c r="D476" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="477" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A477" s="1" t="n">
+        <v>627</v>
+      </c>
+      <c r="B477" s="1" t="s">
+        <v>967</v>
+      </c>
+      <c r="C477" s="1" t="s">
+        <v>968</v>
+      </c>
+      <c r="D477" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="478" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A478" s="1" t="n">
+        <v>628</v>
+      </c>
+      <c r="B478" s="1" t="s">
+        <v>969</v>
+      </c>
+      <c r="C478" s="1" t="s">
+        <v>970</v>
+      </c>
+      <c r="D478" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="479" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A479" s="1" t="n">
+        <v>629</v>
+      </c>
+      <c r="B479" s="1" t="s">
+        <v>971</v>
+      </c>
+      <c r="C479" s="1" t="s">
+        <v>972</v>
+      </c>
+      <c r="D479" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="480" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A480" s="1" t="n">
+        <v>630</v>
+      </c>
+      <c r="B480" s="1" t="s">
+        <v>973</v>
+      </c>
+      <c r="C480" s="1" t="s">
+        <v>974</v>
+      </c>
+      <c r="D480" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="481" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A481" s="1" t="n">
+        <v>631</v>
+      </c>
+      <c r="B481" s="1" t="s">
+        <v>975</v>
+      </c>
+      <c r="C481" s="1" t="s">
+        <v>976</v>
+      </c>
+      <c r="D481" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="482" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A482" s="1" t="n">
+        <v>632</v>
+      </c>
+      <c r="B482" s="1" t="s">
+        <v>977</v>
+      </c>
+      <c r="C482" s="1" t="s">
+        <v>978</v>
+      </c>
+      <c r="D482" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="483" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A483" s="1" t="n">
+        <v>633</v>
+      </c>
+      <c r="B483" s="1" t="s">
+        <v>979</v>
+      </c>
+      <c r="C483" s="1" t="s">
+        <v>980</v>
+      </c>
+      <c r="D483" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="484" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A484" s="1" t="n">
+        <v>634</v>
+      </c>
+      <c r="B484" s="1" t="s">
+        <v>981</v>
+      </c>
+      <c r="C484" s="1" t="s">
+        <v>982</v>
+      </c>
+      <c r="D484" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="485" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A485" s="1" t="n">
+        <v>635</v>
+      </c>
+      <c r="B485" s="1" t="s">
+        <v>983</v>
+      </c>
+      <c r="C485" s="1" t="s">
+        <v>984</v>
+      </c>
+      <c r="D485" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="486" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A486" s="1" t="n">
+        <v>636</v>
+      </c>
+      <c r="B486" s="1" t="s">
+        <v>985</v>
+      </c>
+      <c r="C486" s="1" t="s">
+        <v>986</v>
+      </c>
+      <c r="D486" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="487" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A487" s="1" t="n">
+        <v>637</v>
+      </c>
+      <c r="B487" s="1" t="s">
+        <v>987</v>
+      </c>
+      <c r="C487" s="1" t="s">
+        <v>988</v>
+      </c>
+      <c r="D487" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="488" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A488" s="1" t="n">
+        <v>638</v>
+      </c>
+      <c r="B488" s="1" t="s">
+        <v>989</v>
+      </c>
+      <c r="C488" s="1" t="s">
+        <v>990</v>
+      </c>
+      <c r="D488" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="489" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A489" s="1" t="n">
+        <v>639</v>
+      </c>
+      <c r="B489" s="1" t="s">
+        <v>991</v>
+      </c>
+      <c r="C489" s="1" t="s">
+        <v>992</v>
+      </c>
+      <c r="D489" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="490" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A490" s="1" t="n">
+        <v>640</v>
+      </c>
+      <c r="B490" s="1" t="s">
+        <v>993</v>
+      </c>
+      <c r="C490" s="1" t="s">
+        <v>994</v>
+      </c>
+      <c r="D490" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="491" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A491" s="1" t="n">
+        <v>641</v>
+      </c>
+      <c r="B491" s="1" t="s">
+        <v>995</v>
+      </c>
+      <c r="C491" s="1" t="s">
+        <v>996</v>
+      </c>
+      <c r="D491" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="492" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A492" s="1" t="n">
+        <v>642</v>
+      </c>
+      <c r="B492" s="1" t="s">
+        <v>997</v>
+      </c>
+      <c r="C492" s="1" t="s">
+        <v>998</v>
+      </c>
+      <c r="D492" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="493" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A493" s="1" t="n">
+        <v>643</v>
+      </c>
+      <c r="B493" s="1" t="s">
+        <v>999</v>
+      </c>
+      <c r="C493" s="1" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D493" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="494" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A494" s="1" t="n">
+        <v>644</v>
+      </c>
+      <c r="B494" s="1" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C494" s="1" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D494" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="495" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A495" s="1" t="n">
+        <v>645</v>
+      </c>
+      <c r="B495" s="1" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C495" s="1" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D495" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="496" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A496" s="1" t="n">
+        <v>646</v>
+      </c>
+      <c r="B496" s="1" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C496" s="1" t="s">
+        <v>1006</v>
+      </c>
+      <c r="D496" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="497" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A497" s="1" t="n">
+        <v>647</v>
+      </c>
+      <c r="B497" s="1" t="s">
+        <v>1007</v>
+      </c>
+      <c r="C497" s="1" t="s">
+        <v>1008</v>
+      </c>
+      <c r="D497" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="498" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A498" s="1" t="n">
+        <v>648</v>
+      </c>
+      <c r="B498" s="1" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C498" s="1" t="s">
+        <v>1010</v>
+      </c>
+      <c r="D498" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="499" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A499" s="1" t="n">
+        <v>649</v>
+      </c>
+      <c r="B499" s="1" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C499" s="1" t="s">
+        <v>1012</v>
+      </c>
+      <c r="D499" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="500" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A500" s="1" t="n">
+        <v>650</v>
+      </c>
+      <c r="B500" s="1" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C500" s="1" t="s">
+        <v>1014</v>
+      </c>
+      <c r="D500" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="501" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A501" s="1" t="n">
+        <v>651</v>
+      </c>
+      <c r="B501" s="1" t="s">
+        <v>1015</v>
+      </c>
+      <c r="C501" s="1" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D501" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="502" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A502" s="1" t="n">
+        <v>652</v>
+      </c>
+      <c r="B502" s="1" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C502" s="1" t="s">
+        <v>1018</v>
+      </c>
+      <c r="D502" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="503" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A503" s="1" t="n">
+        <v>653</v>
+      </c>
+      <c r="B503" s="1" t="s">
+        <v>1019</v>
+      </c>
+      <c r="C503" s="1" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D503" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="504" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A504" s="1" t="n">
+        <v>654</v>
+      </c>
+      <c r="B504" s="1" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C504" s="1" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D504" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="505" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A505" s="1" t="n">
+        <v>655</v>
+      </c>
+      <c r="B505" s="1" t="s">
+        <v>1023</v>
+      </c>
+      <c r="C505" s="1" t="s">
+        <v>1024</v>
+      </c>
+      <c r="D505" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="506" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A506" s="1" t="n">
+        <v>656</v>
+      </c>
+      <c r="B506" s="1" t="s">
+        <v>1025</v>
+      </c>
+      <c r="C506" s="1" t="s">
+        <v>1026</v>
+      </c>
+      <c r="D506" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="507" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A507" s="1" t="n">
+        <v>657</v>
+      </c>
+      <c r="B507" s="1" t="s">
+        <v>1027</v>
+      </c>
+      <c r="C507" s="1" t="s">
+        <v>1028</v>
+      </c>
+      <c r="D507" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="508" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A508" s="1" t="n">
+        <v>658</v>
+      </c>
+      <c r="B508" s="1" t="s">
+        <v>1029</v>
+      </c>
+      <c r="C508" s="1" t="s">
+        <v>1030</v>
+      </c>
+      <c r="D508" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="509" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A509" s="1" t="n">
+        <v>659</v>
+      </c>
+      <c r="B509" s="1" t="s">
+        <v>1031</v>
+      </c>
+      <c r="C509" s="1" t="s">
+        <v>1032</v>
+      </c>
+      <c r="D509" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="510" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A510" s="1" t="n">
+        <v>660</v>
+      </c>
+      <c r="B510" s="1" t="s">
+        <v>1033</v>
+      </c>
+      <c r="C510" s="1" t="s">
+        <v>1034</v>
+      </c>
+      <c r="D510" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="511" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A511" s="1" t="n">
+        <v>661</v>
+      </c>
+      <c r="B511" s="1" t="s">
+        <v>1035</v>
+      </c>
+      <c r="C511" s="1" t="s">
+        <v>1036</v>
+      </c>
+      <c r="D511" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="512" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A512" s="1" t="n">
+        <v>662</v>
+      </c>
+      <c r="B512" s="1" t="s">
+        <v>1037</v>
+      </c>
+      <c r="C512" s="1" t="s">
+        <v>1038</v>
+      </c>
+      <c r="D512" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="513" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A513" s="1" t="n">
+        <v>663</v>
+      </c>
+      <c r="B513" s="1" t="s">
+        <v>1039</v>
+      </c>
+      <c r="C513" s="1" t="s">
+        <v>1040</v>
+      </c>
+      <c r="D513" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="514" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A514" s="1" t="n">
+        <v>664</v>
+      </c>
+      <c r="B514" s="1" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C514" s="1" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D514" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="515" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A515" s="1" t="n">
+        <v>665</v>
+      </c>
+      <c r="B515" s="1" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C515" s="1" t="s">
+        <v>1044</v>
+      </c>
+      <c r="D515" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="516" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A516" s="1" t="n">
+        <v>666</v>
+      </c>
+      <c r="B516" s="1" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C516" s="1" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D516" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="517" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A517" s="1" t="n">
+        <v>667</v>
+      </c>
+      <c r="B517" s="1" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C517" s="1" t="s">
+        <v>1048</v>
+      </c>
+      <c r="D517" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="518" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A518" s="1" t="n">
+        <v>668</v>
+      </c>
+      <c r="B518" s="1" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C518" s="1" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D518" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="519" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A519" s="1" t="n">
+        <v>669</v>
+      </c>
+      <c r="B519" s="1" t="s">
+        <v>1051</v>
+      </c>
+      <c r="C519" s="1" t="s">
+        <v>1052</v>
+      </c>
+      <c r="D519" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="520" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A520" s="1" t="n">
+        <v>670</v>
+      </c>
+      <c r="B520" s="1" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C520" s="1" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D520" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="521" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A521" s="1" t="n">
+        <v>671</v>
+      </c>
+      <c r="B521" s="1" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C521" s="1" t="s">
+        <v>1056</v>
+      </c>
+      <c r="D521" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="522" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A522" s="1" t="n">
+        <v>672</v>
+      </c>
+      <c r="B522" s="1" t="s">
+        <v>1057</v>
+      </c>
+      <c r="C522" s="1" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D522" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="523" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A523" s="1" t="n">
+        <v>673</v>
+      </c>
+      <c r="B523" s="1" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C523" s="1" t="s">
+        <v>1060</v>
+      </c>
+      <c r="D523" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="524" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A524" s="1" t="n">
+        <v>674</v>
+      </c>
+      <c r="B524" s="1" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C524" s="1" t="s">
+        <v>1062</v>
+      </c>
+      <c r="D524" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="525" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A525" s="1" t="n">
+        <v>675</v>
+      </c>
+      <c r="B525" s="1" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C525" s="1" t="s">
+        <v>1064</v>
+      </c>
+      <c r="D525" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="526" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A526" s="1" t="n">
+        <v>676</v>
+      </c>
+      <c r="B526" s="1" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C526" s="1" t="s">
+        <v>1066</v>
+      </c>
+      <c r="D526" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="527" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A527" s="1" t="n">
+        <v>677</v>
+      </c>
+      <c r="B527" s="1" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C527" s="1" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D527" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="528" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A528" s="1" t="n">
+        <v>678</v>
+      </c>
+      <c r="B528" s="1" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C528" s="1" t="s">
+        <v>1070</v>
+      </c>
+      <c r="D528" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="529" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A529" s="1" t="n">
+        <v>679</v>
+      </c>
+      <c r="B529" s="1" t="s">
+        <v>1071</v>
+      </c>
+      <c r="C529" s="1" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D529" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="530" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A530" s="1" t="n">
+        <v>680</v>
+      </c>
+      <c r="B530" s="1" t="s">
+        <v>1073</v>
+      </c>
+      <c r="C530" s="1" t="s">
+        <v>1074</v>
+      </c>
+      <c r="D530" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="531" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A531" s="1" t="n">
+        <v>681</v>
+      </c>
+      <c r="B531" s="1" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C531" s="1" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D531" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="532" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A532" s="1" t="n">
+        <v>682</v>
+      </c>
+      <c r="B532" s="1" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C532" s="1" t="s">
+        <v>1078</v>
+      </c>
+      <c r="D532" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="533" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A533" s="1" t="n">
+        <v>683</v>
+      </c>
+      <c r="B533" s="1" t="s">
+        <v>1079</v>
+      </c>
+      <c r="C533" s="1" t="s">
+        <v>1080</v>
+      </c>
+      <c r="D533" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="534" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A534" s="1" t="n">
+        <v>684</v>
+      </c>
+      <c r="B534" s="1" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C534" s="1" t="s">
+        <v>1082</v>
+      </c>
+      <c r="D534" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="535" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A535" s="1" t="n">
+        <v>685</v>
+      </c>
+      <c r="B535" s="1" t="s">
+        <v>1083</v>
+      </c>
+      <c r="C535" s="1" t="s">
+        <v>1084</v>
+      </c>
+      <c r="D535" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="536" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A536" s="1" t="n">
+        <v>686</v>
+      </c>
+      <c r="B536" s="1" t="s">
+        <v>1085</v>
+      </c>
+      <c r="C536" s="1" t="s">
+        <v>1086</v>
+      </c>
+      <c r="D536" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="537" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A537" s="1" t="n">
+        <v>687</v>
+      </c>
+      <c r="B537" s="1" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C537" s="1" t="s">
+        <v>1088</v>
+      </c>
+      <c r="D537" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="538" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A538" s="1" t="n">
+        <v>688</v>
+      </c>
+      <c r="B538" s="1" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C538" s="1" t="s">
+        <v>1090</v>
+      </c>
+      <c r="D538" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="539" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A539" s="1" t="n">
+        <v>689</v>
+      </c>
+      <c r="B539" s="1" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C539" s="1" t="s">
+        <v>1092</v>
+      </c>
+      <c r="D539" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="540" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A540" s="1" t="n">
+        <v>690</v>
+      </c>
+      <c r="B540" s="1" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C540" s="1" t="s">
+        <v>1094</v>
+      </c>
+      <c r="D540" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="541" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A541" s="1" t="n">
+        <v>691</v>
+      </c>
+      <c r="B541" s="1" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C541" s="1" t="s">
+        <v>1096</v>
+      </c>
+      <c r="D541" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="542" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A542" s="1" t="n">
+        <v>692</v>
+      </c>
+      <c r="B542" s="1" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C542" s="1" t="s">
+        <v>1098</v>
+      </c>
+      <c r="D542" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="543" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A543" s="1" t="n">
+        <v>693</v>
+      </c>
+      <c r="B543" s="1" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C543" s="1" t="s">
+        <v>1100</v>
+      </c>
+      <c r="D543" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="544" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A544" s="1" t="n">
+        <v>694</v>
+      </c>
+      <c r="B544" s="1" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C544" s="1" t="s">
+        <v>1102</v>
+      </c>
+      <c r="D544" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="545" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A545" s="1" t="n">
+        <v>695</v>
+      </c>
+      <c r="B545" s="1" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C545" s="1" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D545" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="546" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A546" s="1" t="n">
+        <v>696</v>
+      </c>
+      <c r="B546" s="1" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C546" s="1" t="s">
+        <v>1106</v>
+      </c>
+      <c r="D546" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="547" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A547" s="1" t="n">
+        <v>697</v>
+      </c>
+      <c r="B547" s="1" t="s">
+        <v>1107</v>
+      </c>
+      <c r="C547" s="1" t="s">
+        <v>1108</v>
+      </c>
+      <c r="D547" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="548" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A548" s="1" t="n">
+        <v>698</v>
+      </c>
+      <c r="B548" s="1" t="s">
+        <v>1109</v>
+      </c>
+      <c r="C548" s="1" t="s">
+        <v>1110</v>
+      </c>
+      <c r="D548" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="549" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A549" s="1" t="n">
+        <v>699</v>
+      </c>
+      <c r="B549" s="1" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C549" s="1" t="s">
+        <v>1112</v>
+      </c>
+      <c r="D549" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="550" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A550" s="1" t="n">
+        <v>700</v>
+      </c>
+      <c r="B550" s="1" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C550" s="1" t="s">
+        <v>1114</v>
+      </c>
+      <c r="D550" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="551" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A551" s="1" t="n">
+        <v>701</v>
+      </c>
+      <c r="B551" s="1" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C551" s="1" t="s">
+        <v>1116</v>
+      </c>
+      <c r="D551" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="552" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A552" s="1" t="n">
+        <v>702</v>
+      </c>
+      <c r="B552" s="1" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C552" s="1" t="s">
+        <v>1118</v>
+      </c>
+      <c r="D552" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="553" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A553" s="1" t="n">
+        <v>703</v>
+      </c>
+      <c r="B553" s="1" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C553" s="1" t="s">
+        <v>1120</v>
+      </c>
+      <c r="D553" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="554" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A554" s="1" t="n">
+        <v>704</v>
+      </c>
+      <c r="B554" s="1" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C554" s="1" t="s">
+        <v>1122</v>
+      </c>
+      <c r="D554" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="555" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A555" s="1" t="n">
+        <v>705</v>
+      </c>
+      <c r="B555" s="1" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C555" s="1" t="s">
+        <v>1124</v>
+      </c>
+      <c r="D555" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="556" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A556" s="1" t="n">
+        <v>706</v>
+      </c>
+      <c r="B556" s="1" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C556" s="1" t="s">
+        <v>1126</v>
+      </c>
+      <c r="D556" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="557" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A557" s="1" t="n">
+        <v>707</v>
+      </c>
+      <c r="B557" s="1" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C557" s="1" t="s">
+        <v>1128</v>
+      </c>
+      <c r="D557" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="558" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A558" s="1" t="n">
+        <v>708</v>
+      </c>
+      <c r="B558" s="1" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C558" s="1" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D558" s="1" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -10219,16 +12445,16 @@
         <v>3</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>908</v>
+        <v>1131</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>909</v>
+        <v>1132</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>910</v>
+        <v>1133</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>911</v>
+        <v>1134</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>6</v>
@@ -10250,7 +12476,7 @@
         <v>1001</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>912</v>
+        <v>1135</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>13</v>
@@ -10261,7 +12487,7 @@
         <v>1004</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>913</v>
+        <v>1136</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>13</v>
@@ -10272,7 +12498,7 @@
         <v>1005</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>914</v>
+        <v>1137</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>13</v>
@@ -10283,7 +12509,7 @@
         <v>1006</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>915</v>
+        <v>1138</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>13</v>
@@ -10305,7 +12531,7 @@
         <v>1010</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>916</v>
+        <v>1139</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>13</v>
@@ -10316,7 +12542,7 @@
         <v>1011</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>917</v>
+        <v>1140</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>13</v>
@@ -10327,7 +12553,7 @@
         <v>1013</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>918</v>
+        <v>1141</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>13</v>
@@ -10338,7 +12564,7 @@
         <v>1014</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>919</v>
+        <v>1142</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>13</v>
@@ -10349,7 +12575,7 @@
         <v>1015</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>920</v>
+        <v>1143</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>13</v>
@@ -10360,7 +12586,7 @@
         <v>1016</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>921</v>
+        <v>1144</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>13</v>
@@ -10382,7 +12608,7 @@
         <v>1018</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>922</v>
+        <v>1145</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>13</v>
@@ -10393,7 +12619,7 @@
         <v>1019</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>923</v>
+        <v>1146</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>13</v>
@@ -10404,7 +12630,7 @@
         <v>1020</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>924</v>
+        <v>1147</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>13</v>
@@ -10415,7 +12641,7 @@
         <v>1021</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>925</v>
+        <v>1148</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>13</v>
@@ -10426,7 +12652,7 @@
         <v>1022</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>926</v>
+        <v>1149</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>13</v>
@@ -10448,7 +12674,7 @@
         <v>1024</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>927</v>
+        <v>1150</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>13</v>
@@ -10459,7 +12685,7 @@
         <v>1025</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>928</v>
+        <v>1151</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>13</v>
@@ -10470,7 +12696,7 @@
         <v>1026</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>929</v>
+        <v>1152</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>13</v>
@@ -10481,7 +12707,7 @@
         <v>1027</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>930</v>
+        <v>1153</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>13</v>
@@ -10492,7 +12718,7 @@
         <v>1028</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>931</v>
+        <v>1154</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>13</v>
@@ -10503,7 +12729,7 @@
         <v>1029</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>932</v>
+        <v>1155</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>13</v>
@@ -10514,7 +12740,7 @@
         <v>1030</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>933</v>
+        <v>1156</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>13</v>
@@ -10525,7 +12751,7 @@
         <v>1002</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>934</v>
+        <v>1157</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>47</v>
@@ -10536,7 +12762,7 @@
         <v>1003</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>935</v>
+        <v>1158</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>47</v>
@@ -10547,7 +12773,7 @@
         <v>1008</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>936</v>
+        <v>1159</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>47</v>
@@ -10558,7 +12784,7 @@
         <v>1009</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>937</v>
+        <v>1160</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>47</v>
@@ -10569,7 +12795,7 @@
         <v>1012</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>938</v>
+        <v>1161</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>47</v>
@@ -10580,7 +12806,7 @@
         <v>1032</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>939</v>
+        <v>1162</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>47</v>
@@ -10591,7 +12817,7 @@
         <v>1033</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>940</v>
+        <v>1163</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>47</v>
@@ -10602,7 +12828,7 @@
         <v>1034</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>941</v>
+        <v>1164</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>538</v>
@@ -10613,7 +12839,7 @@
         <v>1035</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>942</v>
+        <v>1165</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>538</v>
@@ -10624,7 +12850,7 @@
         <v>1036</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>943</v>
+        <v>1166</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>538</v>
@@ -10635,7 +12861,7 @@
         <v>1037</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>944</v>
+        <v>1167</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>538</v>
@@ -10646,7 +12872,7 @@
         <v>1038</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>945</v>
+        <v>1168</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>538</v>
@@ -10657,7 +12883,7 @@
         <v>1039</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>946</v>
+        <v>1169</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>729</v>
@@ -10673,7 +12899,7 @@
         <v>1040</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>947</v>
+        <v>1170</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>729</v>
@@ -10689,7 +12915,7 @@
         <v>1041</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>948</v>
+        <v>1171</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>729</v>
@@ -10705,7 +12931,7 @@
         <v>1042</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>949</v>
+        <v>1172</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>729</v>
@@ -10721,7 +12947,7 @@
         <v>1043</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>950</v>
+        <v>1173</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>729</v>
@@ -10737,7 +12963,7 @@
         <v>1044</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>951</v>
+        <v>1174</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>729</v>
@@ -10753,7 +12979,7 @@
         <v>1045</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>952</v>
+        <v>1175</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>729</v>
@@ -10769,7 +12995,7 @@
         <v>1046</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>953</v>
+        <v>1176</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>729</v>
@@ -10785,7 +13011,7 @@
         <v>1047</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>954</v>
+        <v>1177</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>729</v>
@@ -10801,7 +13027,7 @@
         <v>1048</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>955</v>
+        <v>1178</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>729</v>
@@ -10817,7 +13043,7 @@
         <v>1049</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>956</v>
+        <v>1179</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>729</v>
@@ -10833,7 +13059,7 @@
         <v>1050</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>957</v>
+        <v>1180</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>729</v>
@@ -10849,7 +13075,7 @@
         <v>1051</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>958</v>
+        <v>1181</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>729</v>
@@ -10901,13 +13127,13 @@
         <v>3</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>908</v>
+        <v>1131</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>909</v>
+        <v>1132</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>959</v>
+        <v>1182</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10915,7 +13141,7 @@
         <v>2000</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>960</v>
+        <v>1183</v>
       </c>
       <c r="C2" s="8" t="s">
         <v>13</v>
@@ -10929,7 +13155,7 @@
         <v>2001</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>961</v>
+        <v>1184</v>
       </c>
       <c r="C3" s="8" t="s">
         <v>13</v>
@@ -10943,7 +13169,7 @@
         <v>2002</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>962</v>
+        <v>1185</v>
       </c>
       <c r="C4" s="8" t="s">
         <v>13</v>
@@ -10957,7 +13183,7 @@
         <v>2013</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>963</v>
+        <v>1186</v>
       </c>
       <c r="C5" s="8" t="s">
         <v>13</v>
@@ -10971,7 +13197,7 @@
         <v>2014</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>964</v>
+        <v>1187</v>
       </c>
       <c r="C6" s="8" t="s">
         <v>13</v>
@@ -10985,7 +13211,7 @@
         <v>2017</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>965</v>
+        <v>1188</v>
       </c>
       <c r="C7" s="8" t="s">
         <v>13</v>
@@ -10999,7 +13225,7 @@
         <v>2010</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>966</v>
+        <v>1189</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>13</v>
@@ -11013,7 +13239,7 @@
         <v>2008</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>967</v>
+        <v>1190</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>13</v>
@@ -11027,7 +13253,7 @@
         <v>2021</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>968</v>
+        <v>1191</v>
       </c>
       <c r="C10" s="8" t="s">
         <v>13</v>
@@ -11041,7 +13267,7 @@
         <v>2022</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>969</v>
+        <v>1192</v>
       </c>
       <c r="C11" s="8" t="s">
         <v>13</v>
@@ -11055,7 +13281,7 @@
         <v>2012</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>970</v>
+        <v>1193</v>
       </c>
       <c r="C12" s="8" t="s">
         <v>13</v>
@@ -11069,7 +13295,7 @@
         <v>2011</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>971</v>
+        <v>1194</v>
       </c>
       <c r="C13" s="8" t="s">
         <v>13</v>
@@ -11083,7 +13309,7 @@
         <v>2015</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>972</v>
+        <v>1195</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>13</v>
@@ -11097,7 +13323,7 @@
         <v>2016</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>973</v>
+        <v>1196</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>13</v>
@@ -11111,7 +13337,7 @@
         <v>2023</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>974</v>
+        <v>1197</v>
       </c>
       <c r="C16" s="8" t="s">
         <v>13</v>
@@ -11125,7 +13351,7 @@
         <v>2024</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>975</v>
+        <v>1198</v>
       </c>
       <c r="C17" s="8" t="s">
         <v>13</v>
@@ -11139,7 +13365,7 @@
         <v>2020</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>976</v>
+        <v>1199</v>
       </c>
       <c r="C18" s="8" t="s">
         <v>47</v>
@@ -11153,7 +13379,7 @@
         <v>2003</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>977</v>
+        <v>1200</v>
       </c>
       <c r="C19" s="8" t="s">
         <v>47</v>
@@ -11167,7 +13393,7 @@
         <v>2004</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>978</v>
+        <v>1201</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>47</v>
@@ -11181,7 +13407,7 @@
         <v>2006</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>979</v>
+        <v>1202</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>47</v>
@@ -11195,7 +13421,7 @@
         <v>2005</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>980</v>
+        <v>1203</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>47</v>
@@ -11209,7 +13435,7 @@
         <v>2018</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>981</v>
+        <v>1204</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>47</v>
@@ -11223,7 +13449,7 @@
         <v>2009</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>982</v>
+        <v>1205</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>47</v>
@@ -11237,7 +13463,7 @@
         <v>2025</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>983</v>
+        <v>1206</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>47</v>
@@ -11251,7 +13477,7 @@
         <v>2007</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>984</v>
+        <v>1207</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>47</v>
@@ -11265,7 +13491,7 @@
         <v>2019</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>985</v>
+        <v>1208</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>47</v>
@@ -11279,7 +13505,7 @@
         <v>2031</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>986</v>
+        <v>1209</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>538</v>
@@ -11293,7 +13519,7 @@
         <v>2030</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>987</v>
+        <v>1210</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>538</v>
@@ -11307,7 +13533,7 @@
         <v>2033</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>988</v>
+        <v>1211</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>538</v>
@@ -11321,7 +13547,7 @@
         <v>2032</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>989</v>
+        <v>1212</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>538</v>
@@ -11335,7 +13561,7 @@
         <v>2026</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>990</v>
+        <v>1213</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>538</v>
@@ -11349,7 +13575,7 @@
         <v>2027</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>991</v>
+        <v>1214</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>538</v>
@@ -11363,7 +13589,7 @@
         <v>2029</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>992</v>
+        <v>1215</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>538</v>
@@ -11377,7 +13603,7 @@
         <v>2028</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>993</v>
+        <v>1216</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>538</v>
@@ -11391,7 +13617,7 @@
         <v>2043</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>994</v>
+        <v>1217</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>729</v>
@@ -11405,7 +13631,7 @@
         <v>2040</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>995</v>
+        <v>1218</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>729</v>
@@ -11419,7 +13645,7 @@
         <v>2035</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>996</v>
+        <v>1219</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>729</v>
@@ -11433,7 +13659,7 @@
         <v>2041</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>997</v>
+        <v>1220</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>729</v>
@@ -11447,7 +13673,7 @@
         <v>2042</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>998</v>
+        <v>1221</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>729</v>
@@ -11461,7 +13687,7 @@
         <v>2044</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>999</v>
+        <v>1222</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>729</v>
@@ -11475,7 +13701,7 @@
         <v>2036</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>1000</v>
+        <v>1223</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>729</v>
@@ -11489,7 +13715,7 @@
         <v>2034</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>1001</v>
+        <v>1224</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>729</v>
@@ -11503,7 +13729,7 @@
         <v>2037</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>1002</v>
+        <v>1225</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>729</v>
@@ -11517,7 +13743,7 @@
         <v>2038</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>1003</v>
+        <v>1226</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>729</v>
@@ -11531,7 +13757,7 @@
         <v>2039</v>
       </c>
       <c r="B46" s="8" t="s">
-        <v>1004</v>
+        <v>1227</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>729</v>
@@ -11545,7 +13771,7 @@
         <v>2045</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>1005</v>
+        <v>1228</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>729</v>
@@ -11584,78 +13810,78 @@
         <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1006</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1007</v>
+        <v>1230</v>
       </c>
       <c r="B2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>1008</v>
+        <v>1231</v>
       </c>
       <c r="B3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>1009</v>
+        <v>1232</v>
       </c>
       <c r="B4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>1010</v>
+        <v>1233</v>
       </c>
       <c r="B5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>1011</v>
+        <v>1234</v>
       </c>
       <c r="B6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>1012</v>
+        <v>1235</v>
       </c>
       <c r="B7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>1013</v>
+        <v>1236</v>
       </c>
       <c r="B8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>1014</v>
+        <v>1237</v>
       </c>
       <c r="B9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>1015</v>
+        <v>1238</v>
       </c>
       <c r="B10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>1016</v>
+        <v>1239</v>
       </c>
       <c r="B11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>1017</v>
+        <v>1240</v>
       </c>
       <c r="B12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>1018</v>
+        <v>1241</v>
       </c>
       <c r="B13" s="2"/>
     </row>
@@ -11691,15 +13917,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>908</v>
+        <v>1131</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>1019</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>1020</v>
+        <v>1243</v>
       </c>
     </row>
   </sheetData>

</xml_diff>